<commit_message>
done update fomula for timeline metrics
</commit_message>
<xml_diff>
--- a/docs/_issue_track.xlsx
+++ b/docs/_issue_track.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA606EE-C0BF-4DCB-AC07-548C51FB03E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8738E8EC-B6F5-406B-89C7-D726AE9D09DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17010" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16320" yWindow="825" windowWidth="16440" windowHeight="27495" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Issue Tracking" sheetId="4" r:id="rId1"/>
@@ -1478,7 +1478,7 @@
         <v>49</v>
       </c>
       <c r="D9" s="48" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E9" s="48" t="s">
         <v>20</v>

</xml_diff>